<commit_message>
feat(rates): Phase A — pincode zone/EDL mapping + EDL matrix (real-format foundation)
Grounded in the uploaded formats (PINCODE MAPPING, EDL Matrix, Rate Updation):
- Pincode enriched with per-product zones (dpZone A/B/C/OTHER, surfaceZone/apexZone
  N1..NE3, ecomZone) + EDL flag + edlDistanceKm + TAT. POST /pincodes/mapping/bulk.
- EdlRate model: standard km-band × weight-band ODA matrix per vendor/network.
  GET /rate-cards/edl, POST /rate-cards/edl/bulk (replace-per-network).
- CustomerRateCardSlab gains originZone (origin×dest grid, faithful to the sheet).
- CustomerRateCard gains the 5 red required fields (min chg wt/freight already present;
  + cityWiseRates, rateAboveKg(+rate), volDiscountPct), handlingBands, ospCharge, and the
  standard surcharge heads (AWB, emergency, environmental).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Formats/Rate Updation format.xlsx
+++ b/Formats/Rate Updation format.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/deeeb9ec8bed1bc2/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://urbanboltin-my.sharepoint.com/personal/jbs_urbanebolt_com/Documents/Apps/Logimart ERP/Formats/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{322B9590-A1CF-47F5-AA86-6448BA47CC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C0985C8-2E5B-49F2-A2BA-7643562CFDF9}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{322B9590-A1CF-47F5-AA86-6448BA47CC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17E276ED-48FE-467C-B304-1863C8ECD36E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6352CA6E-7FE0-4303-98E9-CC76EF6442E3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6352CA6E-7FE0-4303-98E9-CC76EF6442E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Apex And surface" sheetId="1" r:id="rId1"/>
@@ -21,21 +21,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="43">
   <si>
     <t>N1</t>
   </si>
@@ -152,13 +143,25 @@
   </si>
   <si>
     <t>FIRST 250 GM</t>
+  </si>
+  <si>
+    <t>Intracity</t>
+  </si>
+  <si>
+    <t>Within Region</t>
+  </si>
+  <si>
+    <t>Metro</t>
+  </si>
+  <si>
+    <t>ROI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -170,6 +173,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -236,16 +246,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -264,9 +275,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -304,7 +315,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -410,7 +421,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -552,7 +563,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -561,19 +572,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9562ADF4-9D81-4610-8044-01818EF5BFE9}">
   <dimension ref="C3:U37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="44.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C3" s="2" t="s">
+    <row r="3" spans="3:21" x14ac:dyDescent="0.3">
+      <c r="C3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="3"/>
-    </row>
-    <row r="5" spans="3:21" x14ac:dyDescent="0.25">
+      <c r="D3" s="4"/>
+    </row>
+    <row r="5" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
         <v>0</v>
@@ -630,7 +641,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
@@ -653,7 +664,7 @@
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
     </row>
-    <row r="7" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C7" s="1" t="s">
         <v>1</v>
       </c>
@@ -676,7 +687,7 @@
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
     </row>
-    <row r="8" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C8" s="1" t="s">
         <v>2</v>
       </c>
@@ -699,7 +710,7 @@
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
     </row>
-    <row r="9" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
         <v>3</v>
       </c>
@@ -722,7 +733,7 @@
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
     </row>
-    <row r="10" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
         <v>4</v>
       </c>
@@ -745,7 +756,7 @@
       <c r="T10" s="1"/>
       <c r="U10" s="1"/>
     </row>
-    <row r="11" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
@@ -768,7 +779,7 @@
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
     </row>
-    <row r="12" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
         <v>6</v>
       </c>
@@ -791,7 +802,7 @@
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
     </row>
-    <row r="13" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
         <v>7</v>
       </c>
@@ -814,7 +825,7 @@
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
     </row>
-    <row r="14" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C14" s="1" t="s">
         <v>8</v>
       </c>
@@ -837,7 +848,7 @@
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
     </row>
-    <row r="15" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
         <v>9</v>
       </c>
@@ -860,7 +871,7 @@
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
     </row>
-    <row r="16" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
         <v>10</v>
       </c>
@@ -883,7 +894,7 @@
       <c r="T16" s="1"/>
       <c r="U16" s="1"/>
     </row>
-    <row r="17" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
         <v>11</v>
       </c>
@@ -906,7 +917,7 @@
       <c r="T17" s="1"/>
       <c r="U17" s="1"/>
     </row>
-    <row r="18" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
         <v>12</v>
       </c>
@@ -929,7 +940,7 @@
       <c r="T18" s="1"/>
       <c r="U18" s="1"/>
     </row>
-    <row r="19" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C19" s="1" t="s">
         <v>13</v>
       </c>
@@ -952,7 +963,7 @@
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
     </row>
-    <row r="20" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C20" s="1" t="s">
         <v>14</v>
       </c>
@@ -975,7 +986,7 @@
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
     </row>
-    <row r="21" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
         <v>15</v>
       </c>
@@ -998,7 +1009,7 @@
       <c r="T21" s="1"/>
       <c r="U21" s="1"/>
     </row>
-    <row r="22" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C22" s="1" t="s">
         <v>16</v>
       </c>
@@ -1021,7 +1032,7 @@
       <c r="T22" s="1"/>
       <c r="U22" s="1"/>
     </row>
-    <row r="23" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C23" s="1" t="s">
         <v>17</v>
       </c>
@@ -1044,36 +1055,36 @@
       <c r="T23" s="1"/>
       <c r="U23" s="1"/>
     </row>
-    <row r="25" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-    </row>
-    <row r="26" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="D26" t="s">
+    <row r="25" spans="3:21" x14ac:dyDescent="0.3">
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="3:21" x14ac:dyDescent="0.3">
+      <c r="D26" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="D27" t="s">
+    <row r="27" spans="3:21" x14ac:dyDescent="0.3">
+      <c r="D27" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="D28" t="s">
+    <row r="28" spans="3:21" x14ac:dyDescent="0.3">
+      <c r="D28" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="D29" t="s">
+    <row r="29" spans="3:21" x14ac:dyDescent="0.3">
+      <c r="D29" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="3:21" x14ac:dyDescent="0.25">
-      <c r="D30" t="s">
+    <row r="30" spans="3:21" x14ac:dyDescent="0.3">
+      <c r="D30" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:21" x14ac:dyDescent="0.3">
       <c r="D31" t="s">
         <v>23</v>
       </c>
@@ -1084,7 +1095,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="3:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:21" x14ac:dyDescent="0.3">
       <c r="E32" s="1" t="s">
         <v>26</v>
       </c>
@@ -1092,7 +1103,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="4:6" x14ac:dyDescent="0.3">
       <c r="E33" s="1" t="s">
         <v>27</v>
       </c>
@@ -1100,7 +1111,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="4:6" x14ac:dyDescent="0.3">
       <c r="E34" s="1" t="s">
         <v>28</v>
       </c>
@@ -1108,12 +1119,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="4:6" x14ac:dyDescent="0.3">
       <c r="D36" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="37" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="4:6" x14ac:dyDescent="0.3">
       <c r="D37" t="s">
         <v>30</v>
       </c>
@@ -1128,10 +1139,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9975C85F-2FD9-4AE9-956A-A450C21B4B8E}">
-  <dimension ref="A2:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>32</v>
@@ -1146,7 +1174,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>32</v>
       </c>
@@ -1155,7 +1183,7 @@
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>33</v>
       </c>
@@ -1164,7 +1192,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -1173,7 +1201,7 @@
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
@@ -1182,17 +1210,17 @@
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
feat(rates): Phase B2 — rate-matrix uploader (cargo) + 60MB body limit
- Upload UI in the rate-cards popout: ⬆ Upload rates (pick Network + Product, drop the
  filled matrix) + ⬇ blank cargo template. Client-side SheetJS parser auto-detects the
  origin×dest zone matrix by position and reads rate cells → PLUSKG slabs (Apex/Surface).
  Courier (DP/TDD/NDD) matrix is detected but parsing awaits a filled sample.
- xlsx lazy-loaded (own chunk) so the main bundle stays small.
- API body limit raised to 60MB for large bulk uploads (21k-row pincode mapping etc.).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Formats/Rate Updation format.xlsx
+++ b/Formats/Rate Updation format.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://urbanboltin-my.sharepoint.com/personal/jbs_urbanebolt_com/Documents/Apps/Logimart ERP/Formats/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive - Urbanlogix Global India Pvt Ltd\Apps\Logimart ERP\Formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{322B9590-A1CF-47F5-AA86-6448BA47CC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17E276ED-48FE-467C-B304-1863C8ECD36E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E4B03C-F4B0-4905-B89C-56EEE2E02CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6352CA6E-7FE0-4303-98E9-CC76EF6442E3}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="45">
   <si>
     <t>N1</t>
   </si>
@@ -155,6 +155,12 @@
   </si>
   <si>
     <t>ROI</t>
+  </si>
+  <si>
+    <t>Weight Slab</t>
+  </si>
+  <si>
+    <t>Zone</t>
   </si>
 </sst>
 </file>
@@ -193,7 +199,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -242,21 +248,67 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -579,10 +631,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:21" x14ac:dyDescent="0.3">
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="4"/>
+      <c r="D3" s="5"/>
     </row>
     <row r="5" spans="3:21" x14ac:dyDescent="0.3">
       <c r="C5" s="1"/>
@@ -1060,27 +1112,27 @@
       <c r="D25" s="2"/>
     </row>
     <row r="26" spans="3:21" x14ac:dyDescent="0.3">
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="27" spans="3:21" x14ac:dyDescent="0.3">
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="28" spans="3:21" x14ac:dyDescent="0.3">
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="29" spans="3:21" x14ac:dyDescent="0.3">
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="3:21" x14ac:dyDescent="0.3">
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="3" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1139,93 +1191,208 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9975C85F-2FD9-4AE9-956A-A450C21B4B8E}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="1"/>
+        <v>37</v>
+      </c>
+      <c r="B4" s="7"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="1"/>
+        <v>36</v>
+      </c>
+      <c r="B5" s="8"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B7" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="B9" s="8"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="7"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B3:B5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>